<commit_message>
feat: stop silent table truncation, exact Java unsigned types, English headers
- Blank rows are skipped instead of ending the sheet; headers after an empty
  header column are read, and data under an empty header is a located
  DataUnderEmptyHeader error instead of being silently dropped
- XLSX reads no longer grow sheets on out-of-range access
- Java: uint/uint32 map to long, uint64 to BigInteger, so full ranges load
- Index, type and KV tables accept English header names as aliases
- Give the example's note column a #备注 header

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/v3/example/xlsx/Type.xlsx
+++ b/v3/example/xlsx/Type.xlsx
@@ -1171,7 +1171,7 @@
     <col min="5" max="5" width="11.1333333333333" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="16.5" spans="1:9">
+    <row r="1" s="1" customFormat="1" ht="16.5" spans="1:10">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1198,6 +1198,11 @@
       </c>
       <c r="I1" s="2" t="s">
         <v>8</v>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>#备注</t>
+        </is>
       </c>
     </row>
     <row r="2" ht="16.5" spans="1:11">

</xml_diff>